<commit_message>
SSLC 1110 reconciliation: fix sign error, recompute FY27 shortfall + FY26 True-Up revenue quality
</commit_message>
<xml_diff>
--- a/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-11.xlsx
+++ b/drafts/SSLC_QB_Equity_Debt_Microcosm_Facility_2026-10-11.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Facility Costs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Microcosm Offset" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IM tank reconciliation" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +68,57 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -100,8 +150,73 @@
         <fgColor rgb="00FFDCE1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6B6B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -167,11 +282,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -229,6 +358,120 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3269,284 +3512,1382 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="65" t="inlineStr">
+        <is>
+          <t>SIGN-CORRECTION NOTE — PRIOR ANALYSIS HAD SIGN BACKWARDS (added 2026-10-11 revision)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Account 1110 AR Unbilled is an ASSET with a CREDIT (negative) balance. Invoice entries = CREDITS (increase billed-ahead). Rev-rec debits = DEBITS (reduce billed-ahead). The prior reconciliation treated this backwards, computing overstatement as if True-Up JEs increased 1110 rather than reduced it. This section corrects the analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1"/>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>CORRECTED FINDING 1: FY27 REV-REC SHORTFALL — MISSING REVENUE RECOGNITION (Sep–Oct 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>In FY27 (Jul 1 – Oct 11, 2026), SSLC posted 9 IM-109 invoice credits totaling $1,265,282.55 to account 1110 — all growing the billed-ahead balance. Against those, only TWO rev-rec debits appear: 'Unbilled IM' +$545,747 on 7/31/2026 and 'ALC Aug26/013 IM 109-89' +$167,362.41 on 8/31/2026. No Sep or Oct 2026 rev-rec debits exist. Shortfall: $1,265,282.55 − $713,109.41 = $552,173.14. This shortfall is a candidate FY27 overstatement of the billed-ahead balance — meaning SSLC may have shipped tanks in Sep–Oct 2026 without booking the corresponding revenue recognition. [needs SSLC shipping records]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="51" customHeight="1"/>
+    <row r="7" ht="27" customHeight="1">
+      <c r="A7" s="66" t="inlineStr">
+        <is>
+          <t>CORRECTED FINDING 2: 6/30/2026 TRUE-UP JEs — FY26 REVENUE QUALITY ISSUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Three True-Up JEs posted on 6/30/2026 DEBITED account 1110 (reduced billed-ahead) and CREDITED revenue account 4060 — recognizing $515,215.19 of FY26 revenue: IM 122 +$302,988.00, EXOS-133 +$170,530.50, IM 134 +$41,696.69. If these are unsupported (no new PO, no contract amendment, no additional work performed), they overstate FY26 net income by $515,215.19 and understate the true billed-ahead balance. Reversing them: 1110 = −$942,177 − $515,215 = −$1,457,392 (credit). The QB-reported balance of $942,177 would grow to $1,457,392 — meaning SSLC has billed $1.46M ahead of recognized revenue, not $942K. The most material item is IM-122 Nova-D ($302,988) — a program last invoiced 22 months before the True-Up with no visible contract amendment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="67" customHeight="1"/>
+    <row r="10" ht="67" customHeight="1">
+      <c r="A10" s="65" t="inlineStr">
+        <is>
+          <t>CORRECTED FINDING 3: EXOS-133 — $170,531 UNBILLED CLAIM AGAINST EXOS AEROSPACE AS COUNTERPARTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>The EXOS-133 True-Up is not merely an accounting risk — it is an unsupported claim by SSLC against Exos Aerospace specifically. SSLC invoice 133-4 was labeled "Final Balance" on 4/17/2026 and was paid in full by 4/29/2026. Two months later, SSLC booked a $170,530.50 unbilled accrual against the EXOS-133 job, creating a revenue receivable from Exos with no corresponding invoice, no contract amendment, and no Exos acknowledgment visible in the GL. This is an Exos counterparty risk: if SSLC attempts to collect this $170,531, Exos would be receiving an invoice after its own "Final Balance" was paid. Needs immediate contract-amendment check or write-off recommendation in SSLC's books.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1"/>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>OVERSTATEMENT ARITHMETIC (corrected):</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FY27 rev-rec shortfall (IM-109): $552,173.14  [needs SSLC shipping records — candidate only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FY26 True-Up JEs (if unsupported): $515,215.19 → 1110 balance = −$1,457,392 (vs. reported −$942,177)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EXOS-133 component of above: $170,530.50 (Exos counterparty exposure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1"/>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>FACTS vs. INFERENCES:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FACT: IM-109 invoices 109-86/87/88 posted Sep 2026 with no Sep–Oct 2026 rev-rec debits in GL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FACT: True-Up JEs all posted 6/30/2026 with num "True-Up Unbilled" and no PO/invoice reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FACT: Inv 133-4 description reads "Final Balance" (Apr 2026); EXOS-133 True-Up posted 2 months later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="33" customHeight="1">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INFERENCE: True-Up JEs are unsupported and should be reversed — NOT confirmed without SSLC records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  INFERENCE: FY27 shortfall = tanks shipped with no recognition — NOT confirmed without SSLC shipping records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>(PRIOR FINDINGS CONTENT CONTINUES BELOW — NOTE: overstatement math in that section used incorrect sign; see above for corrected figures)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>IM TANK BILLING RECONCILIATION — HYPOTHESIS TEST (Added 2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>John's hypothesis [PARTIALLY CONFIRMED — different mechanism than expected]: Start-billings for IM tanks ARE being relieved through the normal invoice-to-1110-relief JE process. However, three 'True-Up Unbilled' journal entries added at 6/30/2026 total $515,215 and have NO subsequent invoice or relief entry. These accruals — for JN122 (IM Nova-D, $302,988), JN133/EXOS-133 ($170,531), and JN134 (IM T&amp;M, $41,697) — are the primary overstatement risk in 1110.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>WHAT THE DATA SHOWS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Account 1110 (AR Unbilled) QB balance = $942,177 as of 10/11/2026. The GL covers Jan 2024–Oct 2026 with 184 entries. Period net activity = −$395,285; implied beginning balance = $1,337,462 (pre-Jan 2024 accruals).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SSLC billing model: IM tank orders are invoiced on a milestone/progress basis (downpayment → progress → final). Each invoice triggers a negative JE in 1110 (Dr 1100 / Cr 1110), properly relieving the unbilled accrual. Account 2380 (Deposits from Customers) has ZERO IM entries — it is only used for Exos HVRR (and those were reversed). The 'start-billing' mechanism John described does not run through 2380 for IM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>JN109 (active IM program): 35 invoices (109-56 through 109-88, Jan 2025–Sep 2026 = $3.0M+ billed), all properly relieved in 1110. In-progress: +$167,362 (ALC Aug26/013, invoice 109-89 pending). This is legitimate unbilled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>TANKS / JOBS WITH UNRELIEVED OR SUSPECT ACCRUALS:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1. JN122 (IM Nova-D) — $302,988.00 SUSPECT/UNRELIEVED: Original 2024 contract billed 4 invoices ($432,840 total) in Jun–Aug 2024, all collected. 22 months later, a 'True-Up Unbilled' JE of $302,988 was booked 6/30/2026 with no subsequent invoice (no Inv 122-5 found). No completion or shipment language in GL. Nova-D is an IM lunar lander program — if tank work was restarted under a new scope, no contract amendment or invoice is visible. This is the LARGEST suspect item. [NEEDS SSLC contract records and any 2025–2026 work orders for JN122]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2. JN133 / EXOS-133 (HVRR RDRE) — $170,530.50 SUSPECT/UNRELIEVED: Four invoices (133-1 Downpayment, 133-2 Progress #1, 133-3 Progress #2, 133-4 'Final Balance') totaling $211,740 all issued Dec 2025–Apr 2026 and fully paid. A True-Up of $170,530.50 was booked 6/30/2026 — two months AFTER the 'Final Balance' invoice. No subsequent invoice found. The 'Final Balance' language on Inv 133-4 strongly suggests the contract was closed, making this accrual a probable overstatement. [NEEDS SSLC work-order records and any scope-change approvals]</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>3. JN134 (IM T&amp;M Engineering) — $41,696.69 NEEDS RECORDS: Three T&amp;M invoices (134-1/134-2/134-3 = $41,697 total) issued Mar–May 2026 and paid. A True-Up of $41,697 was booked 6/30/2026. A FedEx bill labeled 'IM 134-4' exists dated 2/13/2026 suggesting a delivery. No Inv 134-4 found. Could represent legitimate additional T&amp;M scope or could be a stale accrual. Amount is small but confirms pattern. [NEEDS SSLC T&amp;M logs and any approved extension]</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>OVERSTATEMENT MATH:</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QB 1110 Balance:                           $942,177.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Less JN122 suspect accrual:               −$302,988.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Less JN133/EXOS-133 suspect accrual:     −$170,530.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <f> CONSERVATIVE CORRECTED BALANCE:         $468,658.50  (removes the two most-defensible overstatements)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Less JN134 (needs records):               −$41,696.69</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <f> AGGRESSIVE CORRECTED BALANCE:           $426,961.81  (all three True-Up accruals removed)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Legitimately in-progress (JN109 inv 109-89): $167,362.41 — appropriate to carry</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>WHERE RECORDS ARE INSUFFICIENT:</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>[NEEDS SSLC SHIPPING RECORDS] JN122: No shipment evidence in GL. GL report only covers 2024–2026; older work may not appear. SSLC must provide any 2025–2026 work orders, contract amendments, or IM POs for the Nova-D program to validate or refute the $302,988 True-Up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>[NEEDS SSLC RECORDS] JN133/EXOS-133: Confirm whether any scope-change authorization exists after Inv 133-4 'Final Balance'. If none, the $170,531 is a clear overstatement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>[NEEDS SSLC RECORDS] JN134: Confirm whether T&amp;M authorization extends beyond 134-3 and whether additional T&amp;M charges were approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>BOTTOM LINE FOR DUE DILIGENCE:</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>The mechanism John described (2380-type start-billing deposits not relieved) does not exist for IM — SSLC does not book customer deposits in 2380 for IM. Instead, the risk is $473,519–$515,215 in post-close True-Up accruals booked on 6/30/2026 with no visible contractual basis or subsequent invoicing. The most material item is JN122 IM Nova-D ($302,988) — a program last invoiced 22 months prior. The $942,177 1110 balance as presented is unlikely to be fully collectible. Conservative corrected balance: $468,659. Aggressive: $426,962. The difference ($473K–$515K) represents potential overstatement of current assets in SSLC's balance sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>(END OF IM TANK RECONCILIATION SECTION — existing Findings content continues below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>10/2 → 10/11 Cash Bridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Amount ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Beginning cash (10/2/2026)</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>198419</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>INFLOWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-86 (10/7)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>142605.55</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-87 (10/7)</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>200700</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-88 (10/7)</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>78115</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total AR collections (per GL, EFT1007)</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>421420.55</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>OUTFLOWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vendor payables Bill.com — Hexcel Corp (10/5, JE 270131)</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>-11091.8</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vendor payables Bill.com — Ileana Intl + Stratus (10/6, JE 270135)</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>-3316</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Chase Amazon VISA partial payment (10/5, EFT1005)</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>-10000</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  LACFD permit / hazardous waste (10/2, CK4488)</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>-2452</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Hartford Life insurance (10/8, EFT1008)</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>-1029.56</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Empower 401K + benefits (10/9, EFT1009)</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>-1730.4</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fidelity 401K (10/9, CK4489)</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paychex payroll admin (10/9, EFT1009)</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>-229.39</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total outflows (per GL)</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>-30349.15</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>NET CHANGE PER GL</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>391071.4</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Rounding / beginning-balance adjustment</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>854.05</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Ending cash (10/11/2026)</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>590344.45</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Source: SSLC_Transaction_Detail_by_Account.xlsx (qb-2026-10-11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>All collections from Intuitive Machines (Acct 1100 AR Billed → 1030 Checking).</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>No AR Unbilled (1110) activity between 10/2–10/11 — no new billing-ahead entries recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>$854 rounding gap reflects that stated beginning of $198,419 is rounded; GL-derived net = $391,071.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A19:H19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="28" t="inlineStr">
         <is>
-          <t>10/2 → 10/11 Cash Bridge</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
+          <t>SSLC 1110 AR UNBILLED — CORRECTED RECONCILIATION (SIGN-ERROR FIX)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" s="67" t="inlineStr">
+        <is>
+          <t>Account 1110 is an ASSET with a CREDIT (negative) balance. Invoice entries = CREDITS (make balance more negative). Rev-rec entries = DEBITS (reduce billed-ahead). Prior version had this backwards.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Amount ($)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Beginning cash (10/2/2026)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>198419</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>QB 1110 balance as of 10/11/2026: −$942,177 (credit = billed ahead of revenue)  |  Prepared: 2026-10-11</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-    </row>
-    <row r="6">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>SECTION A: FY27 REV-REC SHORTFALL (IM-109)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
       <c r="A6" s="28" t="inlineStr">
         <is>
-          <t>INFLOWS</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-86 (10/7)</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>142605.55</v>
+          <t>All account 1110 transactions Jul 1 – Oct 11, 2026 (FY27):</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-87 (10/7)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>200700</v>
-      </c>
-    </row>
-    <row r="9">
+      <c r="A8" s="67" t="inlineStr">
+        <is>
+          <t>— IM-109 Invoice Credits (9 entries) —</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  AR Billed collected — Intuitive Machines Inv 109-88 (10/7)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>78115</v>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>270000</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Inv 109-80</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-79179</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total AR collections (per GL, EFT1007)</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>421420.55</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr"/>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>270001</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Inv 109-81</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>-132934</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>270030</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Inv 109-82</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>-132934</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
-        <is>
-          <t>OUTFLOWS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-    </row>
-    <row r="13">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>270035</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Inv 109-83</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>-200700</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vendor payables Bill.com — Hexcel Corp (10/5, JE 270131)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>-11091.8</v>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>270063</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Inv 109-84</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>-78115</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Vendor payables Bill.com — Ileana Intl + Stratus (10/6, JE 270135)</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>-3316</v>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>270064</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Inv 109-85</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>-220000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Chase Amazon VISA partial payment (10/5, EFT1005)</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>-10000</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>270107</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Inv 109-86</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>-142605.55</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  LACFD permit / hazardous waste (10/2, CK4488)</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>-2452</v>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>270108</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Inv 109-87</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>-200700</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Hartford Life insurance (10/8, EFT1008)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>-1029.56</v>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>270132</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Inv 109-88</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Invoice credit</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>-78115</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Billed-ahead grows</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Empower 401K + benefits (10/9, EFT1009)</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>-1730.4</v>
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>— IM-109 Rev-Rec Debits (2 entries) —</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Fidelity 401K (10/9, CK4489)</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>-500</v>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Unbilled</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>IM (Unbilled IM)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Rev-rec debit</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>545747</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Billed-ahead reduces</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Paychex payroll admin (10/9, EFT1009)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>-229.39</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Total outflows (per GL)</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>-30349.15</v>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ALC Aug26/013</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>IM 109-89</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Rev-rec debit</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>167362.41</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Billed-ahead reduces</t>
+        </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Arithmetic:</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t>NET CHANGE PER GL</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>391071.4</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>IM-109 invoice credits posted FY27 (absolute value)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1265282.55</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rounding / beginning-balance adjustment</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>854.05</v>
+          <t>IM-109 rev-rec debits posted FY27</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>713109.41</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr"/>
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Shortfall (billed-ahead grew by, FY27 net) = $1,265,282.55 − $713,109.41</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="n">
+        <v>552173.14</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
-        <is>
-          <t>Ending cash (10/11/2026)</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>590344.45</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="28" t="inlineStr"/>
-      <c r="B27" t="inlineStr"/>
+      <c r="A26" s="67" t="inlineStr">
+        <is>
+          <t>NOTE: Shortfall = candidate FY27 overstatement only IF those tanks were completed/shipped. Sep–Oct 2026 show NO rev-rec debits (invoices 109-86/87/88 posted but no corresponding recognition). [needs SSLC shipping records]</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>NOTES</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="A28" s="66" t="inlineStr">
+        <is>
+          <t>SECTION B: 6/30/2026 TRUE-UP JEs — FY26 REVENUE QUALITY</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Source: SSLC_Transaction_Detail_by_Account.xlsx (qb-2026-10-11)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>These three JEs are DEBITS to 1110 (reduced billed-ahead) and CREDITS to revenue (4060) — they recognized $515,215.19 of revenue in FY26 (fiscal year ending 6/30/2026). If unsupported, they overstate FY26 revenue.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>All collections from Intuitive Machines (Acct 1100 AR Billed → 1030 Checking).</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>Job/Description</t>
+        </is>
+      </c>
+      <c r="D30" s="28" t="inlineStr">
+        <is>
+          <t>Amount (Debit to 1110)</t>
+        </is>
+      </c>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>Supporting evidence in GL</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>No AR Unbilled (1110) activity between 10/2–10/11 — no new billing-ahead entries recorded.</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>True-Up Unbilled</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>IM 122 (Nova-D)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>302988</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>None found — no Inv 122-5, no work-order, 22 months since last invoice</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>SUSPECT — no PO/amendment</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>$854 rounding gap reflects that stated beginning of $198,419 is rounded; GL-derived net = $391,071.</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>True-Up Unbilled</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>EXOS-133 (Exos Aerospace)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>170530.5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>None found — Inv 133-4 labeled 'Final Balance' Apr 2026</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>FLAG — see Section C</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>True-Up Unbilled</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>IM 134 (T&amp;M Eng.)</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>41696.69</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>None found — no Inv 134-4 in GL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NEEDS RECORDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="28" t="inlineStr">
+        <is>
+          <t>Total True-Up JEs (all three):</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="n">
+        <v>515215.19</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>If all three reversed:</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1110 balance = −$942,177 − $515,215.19 = −$1,457,392.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FY26 revenue overstated by: $515,215.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (vs. QB-reported billed-ahead balance of $942,177 — true billed-ahead would be $1,457,392)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="65" t="inlineStr">
+        <is>
+          <t>SECTION C: EXOS-133 FLAG — UNBILLED CLAIM AGAINST EXOS AEROSPACE AS COUNTERPARTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="68" t="inlineStr">
+        <is>
+          <t>SSLC has accrued $170,530.50 as unbilled revenue against Exos Aerospace (EXOS-133 job) after invoice 133-4 was labeled "Final Balance" (Apr 2026). This True-Up JE posted 6/30/2026 — two months after the contract was apparently closed — creates an unsupported claim against a related counterparty. This is not a passive GL entry: it represents $170,531 that SSLC believes it is owed by Exos but has not invoiced. Needs contract amendment, Exos acknowledgment, or write-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="66" t="inlineStr">
+        <is>
+          <t>SECTION D: SUMMARY OF OVERSTATEMENT EFFECTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28" t="inlineStr">
+        <is>
+          <t>Effect</t>
+        </is>
+      </c>
+      <c r="B45" s="28" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C45" s="28" t="inlineStr">
+        <is>
+          <t>Certainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>FY27 rev-rec shortfall (IM-109, if tanks shipped Sep–Oct 2026)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>$552,173.14</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>[needs SSLC shipping records]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>FY26 revenue overstatement (True-Up JEs, if unsupported)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>$515,215.19</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Needs POs/amendments</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  — of which: EXOS-133 (unbilled claim vs. Exos Aerospace)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>$170,530.50</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Flag for Exos review</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>True billed-ahead if True-Ups reversed (vs. QB reported $942,177)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>$1,457,392.19</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Arithmetic — subject to True-Up validity</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A8:H8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>